<commit_message>
Fix dashboard formula bugs: KPI refs, monthly totals, expense category totals, income G column
</commit_message>
<xml_diff>
--- a/Freelancer_Finance_Dashboard.xlsx
+++ b/Freelancer_Finance_Dashboard.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -113,6 +113,66 @@
       <color rgb="00D4A843"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF0F1B33"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF1B2A4A"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF27AE60"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFE74C3C"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF1B2A4A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFD4A843"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -168,7 +228,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -226,6 +286,33 @@
     <xf numFmtId="165" fontId="14" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="18" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="19" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="24" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="24" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -982,8 +1069,9 @@
       <c r="F4" s="14" t="n">
         <v>5000</v>
       </c>
-      <c r="G4" s="14" t="n">
-        <v>0</v>
+      <c r="G4" s="14">
+        <f>IF(F4="","",F4*0.05)</f>
+        <v/>
       </c>
       <c r="H4" s="14">
         <f>F4-G4</f>
@@ -1022,8 +1110,9 @@
       <c r="F5" s="16" t="n">
         <v>3500</v>
       </c>
-      <c r="G5" s="16" t="n">
-        <v>175</v>
+      <c r="G5" s="16">
+        <f>IF(F5="","",F5*0.05)</f>
+        <v/>
       </c>
       <c r="H5" s="16">
         <f>F5-G5</f>
@@ -1062,8 +1151,9 @@
       <c r="F6" s="14" t="n">
         <v>5000</v>
       </c>
-      <c r="G6" s="14" t="n">
-        <v>0</v>
+      <c r="G6" s="14">
+        <f>IF(F6="","",F6*0.05)</f>
+        <v/>
       </c>
       <c r="H6" s="14">
         <f>F6-G6</f>
@@ -1102,8 +1192,9 @@
       <c r="F7" s="16" t="n">
         <v>2800</v>
       </c>
-      <c r="G7" s="16" t="n">
-        <v>140</v>
+      <c r="G7" s="16">
+        <f>IF(F7="","",F7*0.05)</f>
+        <v/>
       </c>
       <c r="H7" s="16">
         <f>F7-G7</f>
@@ -1142,8 +1233,9 @@
       <c r="F8" s="14" t="n">
         <v>1500</v>
       </c>
-      <c r="G8" s="14" t="n">
-        <v>0</v>
+      <c r="G8" s="14">
+        <f>IF(F8="","",F8*0.05)</f>
+        <v/>
       </c>
       <c r="H8" s="14">
         <f>F8-G8</f>
@@ -4241,7 +4333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:I52"/>
+  <dimension ref="B2:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -4257,7 +4349,7 @@
   </cols>
   <sheetData>
     <row r="2">
-      <c r="B2" s="20" t="inlineStr">
+      <c r="B2" s="37" t="inlineStr">
         <is>
           <t>Freelancer Finance Dashboard</t>
         </is>
@@ -4271,83 +4363,83 @@
       <c r="I2" s="21" t="n"/>
     </row>
     <row r="4">
-      <c r="B4" s="22" t="inlineStr">
+      <c r="B4" s="38" t="inlineStr">
         <is>
           <t>Total Income</t>
         </is>
       </c>
-      <c r="C4" s="22" t="inlineStr">
+      <c r="C4" s="38" t="inlineStr">
         <is>
           <t>Total Expenses</t>
         </is>
       </c>
-      <c r="D4" s="22" t="inlineStr">
+      <c r="D4" s="38" t="inlineStr">
         <is>
           <t>Net Profit</t>
         </is>
       </c>
-      <c r="E4" s="22" t="inlineStr">
+      <c r="E4" s="38" t="inlineStr">
         <is>
           <t>Profit Margin</t>
         </is>
       </c>
-      <c r="F4" s="22" t="inlineStr">
+      <c r="F4" s="38" t="inlineStr">
         <is>
           <t>Tax Deductions</t>
         </is>
       </c>
-      <c r="G4" s="22" t="inlineStr">
+      <c r="G4" s="38" t="inlineStr">
         <is>
           <t>Est. Tax Due</t>
         </is>
       </c>
-      <c r="H4" s="22" t="inlineStr">
+      <c r="H4" s="38" t="inlineStr">
         <is>
           <t>Quarterly Payment</t>
         </is>
       </c>
-      <c r="I4" s="22" t="inlineStr">
+      <c r="I4" s="38" t="inlineStr">
         <is>
           <t>After-Tax Income</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="23">
-        <f>SUM(Income!H4:H53)</f>
-        <v/>
-      </c>
-      <c r="C5" s="23">
-        <f>SUM(Expenses!F4:F103)</f>
-        <v/>
-      </c>
-      <c r="D5" s="24">
-        <f>B5-B6</f>
-        <v/>
-      </c>
-      <c r="E5" s="25">
-        <f>IF(B5=0,0,B7/B5)</f>
-        <v/>
-      </c>
-      <c r="F5" s="23">
-        <f>SUM(Expenses!H4:H103)</f>
-        <v/>
-      </c>
-      <c r="G5" s="26">
-        <f>IF(B7&lt;=0,0,B7*0.9235*0.153+MAX(0,B7-11600)*0.12+IF(B7&gt;47150,(B7-47150)*0.1,0))</f>
-        <v/>
-      </c>
-      <c r="H5" s="23">
-        <f>B8/4</f>
-        <v/>
-      </c>
-      <c r="I5" s="24">
-        <f>B7-B8</f>
+      <c r="B5" s="39">
+        <f>SUM(Income!H4:H8)+SUM(Income!H10:H53)</f>
+        <v/>
+      </c>
+      <c r="C5" s="39">
+        <f>SUM(Expenses!F4:F13)+SUM(Expenses!F15:F103)</f>
+        <v/>
+      </c>
+      <c r="D5" s="40">
+        <f>B5-C5</f>
+        <v/>
+      </c>
+      <c r="E5" s="41">
+        <f>IF(B5=0,0,D5/B5)</f>
+        <v/>
+      </c>
+      <c r="F5" s="39">
+        <f>SUM(Expenses!H4:H13)+SUM(Expenses!H15:H103)</f>
+        <v/>
+      </c>
+      <c r="G5" s="42">
+        <f>IF(D5&lt;=0,0,D5*0.9235*0.153+MAX(0,D5-11600)*0.12+IF(D5&gt;47150,(D5-47150)*0.1,0))</f>
+        <v/>
+      </c>
+      <c r="H5" s="39">
+        <f>G5/4</f>
+        <v/>
+      </c>
+      <c r="I5" s="40">
+        <f>D5-G5</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="27" t="inlineStr">
+      <c r="B8" s="43" t="inlineStr">
         <is>
           <t>Monthly Income &amp; Expense Summary</t>
         </is>
@@ -4359,28 +4451,27 @@
       <c r="G8" s="17" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="n"/>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="44" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="C9" s="12" t="inlineStr">
+      <c r="C9" s="44" t="inlineStr">
         <is>
           <t>Income</t>
         </is>
       </c>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="D9" s="44" t="inlineStr">
         <is>
           <t>Expenses</t>
         </is>
       </c>
-      <c r="E9" s="12" t="inlineStr">
+      <c r="E9" s="44" t="inlineStr">
         <is>
           <t>Net Profit</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="44" t="inlineStr">
         <is>
           <t>Cumulative</t>
         </is>
@@ -4393,11 +4484,11 @@
         </is>
       </c>
       <c r="C10" s="14">
-        <f>SUMPRODUCT((MONTH(Income!$B$4:$B$53)=1)*(Income!$H$4:$H$53))</f>
+        <f>SUMPRODUCT((MONTH(Income!$B$4:$B$8)=1)*(Income!$H$4:$H$8))+SUMPRODUCT((MONTH(Income!$B$10:$B$53)=1)*(Income!$H$10:$H$53))</f>
         <v/>
       </c>
       <c r="D10" s="14">
-        <f>SUMPRODUCT((MONTH(Expenses!$B$4:$B$103)=1)*(Expenses!$F$4:$F$103))</f>
+        <f>SUMPRODUCT((MONTH(Expenses!$B$4:$B$13)=1)*(Expenses!$F$4:$F$13))+SUMPRODUCT((MONTH(Expenses!$B$15:$B$103)=1)*(Expenses!$F$15:$F$103))</f>
         <v/>
       </c>
       <c r="E10" s="14">
@@ -4416,11 +4507,11 @@
         </is>
       </c>
       <c r="C11" s="16">
-        <f>SUMPRODUCT((MONTH(Income!$B$4:$B$53)=2)*(Income!$H$4:$H$53))</f>
+        <f>SUMPRODUCT((MONTH(Income!$B$4:$B$8)=2)*(Income!$H$4:$H$8))+SUMPRODUCT((MONTH(Income!$B$10:$B$53)=2)*(Income!$H$10:$H$53))</f>
         <v/>
       </c>
       <c r="D11" s="16">
-        <f>SUMPRODUCT((MONTH(Expenses!$B$4:$B$103)=2)*(Expenses!$F$4:$F$103))</f>
+        <f>SUMPRODUCT((MONTH(Expenses!$B$4:$B$13)=2)*(Expenses!$F$4:$F$13))+SUMPRODUCT((MONTH(Expenses!$B$15:$B$103)=2)*(Expenses!$F$15:$F$103))</f>
         <v/>
       </c>
       <c r="E11" s="16">
@@ -4439,11 +4530,11 @@
         </is>
       </c>
       <c r="C12" s="14">
-        <f>SUMPRODUCT((MONTH(Income!$B$4:$B$53)=3)*(Income!$H$4:$H$53))</f>
+        <f>SUMPRODUCT((MONTH(Income!$B$4:$B$8)=3)*(Income!$H$4:$H$8))+SUMPRODUCT((MONTH(Income!$B$10:$B$53)=3)*(Income!$H$10:$H$53))</f>
         <v/>
       </c>
       <c r="D12" s="14">
-        <f>SUMPRODUCT((MONTH(Expenses!$B$4:$B$103)=3)*(Expenses!$F$4:$F$103))</f>
+        <f>SUMPRODUCT((MONTH(Expenses!$B$4:$B$13)=3)*(Expenses!$F$4:$F$13))+SUMPRODUCT((MONTH(Expenses!$B$15:$B$103)=3)*(Expenses!$F$15:$F$103))</f>
         <v/>
       </c>
       <c r="E12" s="14">
@@ -4462,11 +4553,11 @@
         </is>
       </c>
       <c r="C13" s="16">
-        <f>SUMPRODUCT((MONTH(Income!$B$4:$B$53)=4)*(Income!$H$4:$H$53))</f>
+        <f>SUMPRODUCT((MONTH(Income!$B$4:$B$8)=4)*(Income!$H$4:$H$8))+SUMPRODUCT((MONTH(Income!$B$10:$B$53)=4)*(Income!$H$10:$H$53))</f>
         <v/>
       </c>
       <c r="D13" s="16">
-        <f>SUMPRODUCT((MONTH(Expenses!$B$4:$B$103)=4)*(Expenses!$F$4:$F$103))</f>
+        <f>SUMPRODUCT((MONTH(Expenses!$B$4:$B$13)=4)*(Expenses!$F$4:$F$13))+SUMPRODUCT((MONTH(Expenses!$B$15:$B$103)=4)*(Expenses!$F$15:$F$103))</f>
         <v/>
       </c>
       <c r="E13" s="16">
@@ -4485,11 +4576,11 @@
         </is>
       </c>
       <c r="C14" s="14">
-        <f>SUMPRODUCT((MONTH(Income!$B$4:$B$53)=5)*(Income!$H$4:$H$53))</f>
+        <f>SUMPRODUCT((MONTH(Income!$B$4:$B$8)=5)*(Income!$H$4:$H$8))+SUMPRODUCT((MONTH(Income!$B$10:$B$53)=5)*(Income!$H$10:$H$53))</f>
         <v/>
       </c>
       <c r="D14" s="14">
-        <f>SUMPRODUCT((MONTH(Expenses!$B$4:$B$103)=5)*(Expenses!$F$4:$F$103))</f>
+        <f>SUMPRODUCT((MONTH(Expenses!$B$4:$B$13)=5)*(Expenses!$F$4:$F$13))+SUMPRODUCT((MONTH(Expenses!$B$15:$B$103)=5)*(Expenses!$F$15:$F$103))</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -4508,11 +4599,11 @@
         </is>
       </c>
       <c r="C15" s="16">
-        <f>SUMPRODUCT((MONTH(Income!$B$4:$B$53)=6)*(Income!$H$4:$H$53))</f>
+        <f>SUMPRODUCT((MONTH(Income!$B$4:$B$8)=6)*(Income!$H$4:$H$8))+SUMPRODUCT((MONTH(Income!$B$10:$B$53)=6)*(Income!$H$10:$H$53))</f>
         <v/>
       </c>
       <c r="D15" s="16">
-        <f>SUMPRODUCT((MONTH(Expenses!$B$4:$B$103)=6)*(Expenses!$F$4:$F$103))</f>
+        <f>SUMPRODUCT((MONTH(Expenses!$B$4:$B$13)=6)*(Expenses!$F$4:$F$13))+SUMPRODUCT((MONTH(Expenses!$B$15:$B$103)=6)*(Expenses!$F$15:$F$103))</f>
         <v/>
       </c>
       <c r="E15" s="16">
@@ -4531,11 +4622,11 @@
         </is>
       </c>
       <c r="C16" s="14">
-        <f>SUMPRODUCT((MONTH(Income!$B$4:$B$53)=7)*(Income!$H$4:$H$53))</f>
+        <f>SUMPRODUCT((MONTH(Income!$B$4:$B$8)=7)*(Income!$H$4:$H$8))+SUMPRODUCT((MONTH(Income!$B$10:$B$53)=7)*(Income!$H$10:$H$53))</f>
         <v/>
       </c>
       <c r="D16" s="14">
-        <f>SUMPRODUCT((MONTH(Expenses!$B$4:$B$103)=7)*(Expenses!$F$4:$F$103))</f>
+        <f>SUMPRODUCT((MONTH(Expenses!$B$4:$B$13)=7)*(Expenses!$F$4:$F$13))+SUMPRODUCT((MONTH(Expenses!$B$15:$B$103)=7)*(Expenses!$F$15:$F$103))</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -4554,11 +4645,11 @@
         </is>
       </c>
       <c r="C17" s="16">
-        <f>SUMPRODUCT((MONTH(Income!$B$4:$B$53)=8)*(Income!$H$4:$H$53))</f>
+        <f>SUMPRODUCT((MONTH(Income!$B$4:$B$8)=8)*(Income!$H$4:$H$8))+SUMPRODUCT((MONTH(Income!$B$10:$B$53)=8)*(Income!$H$10:$H$53))</f>
         <v/>
       </c>
       <c r="D17" s="16">
-        <f>SUMPRODUCT((MONTH(Expenses!$B$4:$B$103)=8)*(Expenses!$F$4:$F$103))</f>
+        <f>SUMPRODUCT((MONTH(Expenses!$B$4:$B$13)=8)*(Expenses!$F$4:$F$13))+SUMPRODUCT((MONTH(Expenses!$B$15:$B$103)=8)*(Expenses!$F$15:$F$103))</f>
         <v/>
       </c>
       <c r="E17" s="16">
@@ -4577,11 +4668,11 @@
         </is>
       </c>
       <c r="C18" s="14">
-        <f>SUMPRODUCT((MONTH(Income!$B$4:$B$53)=9)*(Income!$H$4:$H$53))</f>
+        <f>SUMPRODUCT((MONTH(Income!$B$4:$B$8)=9)*(Income!$H$4:$H$8))+SUMPRODUCT((MONTH(Income!$B$10:$B$53)=9)*(Income!$H$10:$H$53))</f>
         <v/>
       </c>
       <c r="D18" s="14">
-        <f>SUMPRODUCT((MONTH(Expenses!$B$4:$B$103)=9)*(Expenses!$F$4:$F$103))</f>
+        <f>SUMPRODUCT((MONTH(Expenses!$B$4:$B$13)=9)*(Expenses!$F$4:$F$13))+SUMPRODUCT((MONTH(Expenses!$B$15:$B$103)=9)*(Expenses!$F$15:$F$103))</f>
         <v/>
       </c>
       <c r="E18" s="14">
@@ -4600,11 +4691,11 @@
         </is>
       </c>
       <c r="C19" s="16">
-        <f>SUMPRODUCT((MONTH(Income!$B$4:$B$53)=10)*(Income!$H$4:$H$53))</f>
+        <f>SUMPRODUCT((MONTH(Income!$B$4:$B$8)=10)*(Income!$H$4:$H$8))+SUMPRODUCT((MONTH(Income!$B$10:$B$53)=10)*(Income!$H$10:$H$53))</f>
         <v/>
       </c>
       <c r="D19" s="16">
-        <f>SUMPRODUCT((MONTH(Expenses!$B$4:$B$103)=10)*(Expenses!$F$4:$F$103))</f>
+        <f>SUMPRODUCT((MONTH(Expenses!$B$4:$B$13)=10)*(Expenses!$F$4:$F$13))+SUMPRODUCT((MONTH(Expenses!$B$15:$B$103)=10)*(Expenses!$F$15:$F$103))</f>
         <v/>
       </c>
       <c r="E19" s="16">
@@ -4623,11 +4714,11 @@
         </is>
       </c>
       <c r="C20" s="14">
-        <f>SUMPRODUCT((MONTH(Income!$B$4:$B$53)=11)*(Income!$H$4:$H$53))</f>
+        <f>SUMPRODUCT((MONTH(Income!$B$4:$B$8)=11)*(Income!$H$4:$H$8))+SUMPRODUCT((MONTH(Income!$B$10:$B$53)=11)*(Income!$H$10:$H$53))</f>
         <v/>
       </c>
       <c r="D20" s="14">
-        <f>SUMPRODUCT((MONTH(Expenses!$B$4:$B$103)=11)*(Expenses!$F$4:$F$103))</f>
+        <f>SUMPRODUCT((MONTH(Expenses!$B$4:$B$13)=11)*(Expenses!$F$4:$F$13))+SUMPRODUCT((MONTH(Expenses!$B$15:$B$103)=11)*(Expenses!$F$15:$F$103))</f>
         <v/>
       </c>
       <c r="E20" s="14">
@@ -4646,11 +4737,11 @@
         </is>
       </c>
       <c r="C21" s="16">
-        <f>SUMPRODUCT((MONTH(Income!$B$4:$B$53)=12)*(Income!$H$4:$H$53))</f>
+        <f>SUMPRODUCT((MONTH(Income!$B$4:$B$8)=12)*(Income!$H$4:$H$8))+SUMPRODUCT((MONTH(Income!$B$10:$B$53)=12)*(Income!$H$10:$H$53))</f>
         <v/>
       </c>
       <c r="D21" s="16">
-        <f>SUMPRODUCT((MONTH(Expenses!$B$4:$B$103)=12)*(Expenses!$F$4:$F$103))</f>
+        <f>SUMPRODUCT((MONTH(Expenses!$B$4:$B$13)=12)*(Expenses!$F$4:$F$13))+SUMPRODUCT((MONTH(Expenses!$B$15:$B$103)=12)*(Expenses!$F$15:$F$103))</f>
         <v/>
       </c>
       <c r="E21" s="16">
@@ -4663,30 +4754,30 @@
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="28" t="inlineStr">
+      <c r="B22" s="45" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C22" s="29">
+      <c r="C22" s="46">
+        <f>SUM(C10:C21)</f>
+        <v/>
+      </c>
+      <c r="D22" s="46">
         <f>SUM(D10:D21)</f>
         <v/>
       </c>
-      <c r="D22" s="29">
+      <c r="E22" s="46">
         <f>SUM(E10:E21)</f>
         <v/>
       </c>
-      <c r="E22" s="29">
-        <f>SUM(F10:F21)</f>
-        <v/>
-      </c>
-      <c r="F22" s="29">
-        <f>SUM(G10:G21)</f>
+      <c r="F22" s="46">
+        <f>F21</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="27" t="inlineStr">
+      <c r="B24" s="43" t="inlineStr">
         <is>
           <t>Expense Breakdown by Category</t>
         </is>
@@ -4696,36 +4787,35 @@
       <c r="E24" s="17" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="n"/>
-      <c r="B25" s="12" t="inlineStr">
+      <c r="B25" s="44" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="C25" s="12" t="inlineStr">
+      <c r="C25" s="44" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="D25" s="12" t="inlineStr">
+      <c r="D25" s="44" t="inlineStr">
         <is>
           <t>% of Total</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E25" s="44" t="inlineStr">
         <is>
           <t>Deductible</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B26" s="47" t="inlineStr">
         <is>
           <t>Office Supplies</t>
         </is>
       </c>
       <c r="C26" s="30">
-        <f>SUMPRODUCT((Expenses!$D$4:$D$103="Office Supplies")*Expenses!$F$4:$F$103)</f>
+        <f>SUMPRODUCT((Expenses!$D$4:$D$13="Office Supplies")*Expenses!$F$4:$F$13)+SUMPRODUCT((Expenses!$D$15:$D$103="Office Supplies")*Expenses!$F$15:$F$103)</f>
         <v/>
       </c>
       <c r="D26" s="31">
@@ -4733,18 +4823,18 @@
         <v/>
       </c>
       <c r="E26" s="30">
-        <f>SUMPRODUCT((Expenses!$D$4:$D$103="Office Supplies")*Expenses!$H$4:$H$103)</f>
+        <f>SUMPRODUCT((Expenses!$D$4:$D$13="Office Supplies")*Expenses!$H$4:$H$13)+SUMPRODUCT((Expenses!$D$15:$D$103="Office Supplies")*Expenses!$H$15:$H$103)</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="7" t="inlineStr">
+      <c r="B27" s="48" t="inlineStr">
         <is>
           <t>Home Office</t>
         </is>
       </c>
       <c r="C27" s="32">
-        <f>SUMPRODUCT((Expenses!$D$4:$D$103="Home Office")*Expenses!$F$4:$F$103)</f>
+        <f>SUMPRODUCT((Expenses!$D$4:$D$13="Home Office")*Expenses!$F$4:$F$13)+SUMPRODUCT((Expenses!$D$15:$D$103="Home Office")*Expenses!$F$15:$F$103)</f>
         <v/>
       </c>
       <c r="D27" s="33">
@@ -4752,18 +4842,18 @@
         <v/>
       </c>
       <c r="E27" s="32">
-        <f>SUMPRODUCT((Expenses!$D$4:$D$103="Home Office")*Expenses!$H$4:$H$103)</f>
+        <f>SUMPRODUCT((Expenses!$D$4:$D$13="Home Office")*Expenses!$H$4:$H$13)+SUMPRODUCT((Expenses!$D$15:$D$103="Home Office")*Expenses!$H$15:$H$103)</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B28" s="47" t="inlineStr">
         <is>
           <t>Travel</t>
         </is>
       </c>
       <c r="C28" s="30">
-        <f>SUMPRODUCT((Expenses!$D$4:$D$103="Travel")*Expenses!$F$4:$F$103)</f>
+        <f>SUMPRODUCT((Expenses!$D$4:$D$13="Travel")*Expenses!$F$4:$F$13)+SUMPRODUCT((Expenses!$D$15:$D$103="Travel")*Expenses!$F$15:$F$103)</f>
         <v/>
       </c>
       <c r="D28" s="31">
@@ -4771,18 +4861,18 @@
         <v/>
       </c>
       <c r="E28" s="30">
-        <f>SUMPRODUCT((Expenses!$D$4:$D$103="Travel")*Expenses!$H$4:$H$103)</f>
+        <f>SUMPRODUCT((Expenses!$D$4:$D$13="Travel")*Expenses!$H$4:$H$13)+SUMPRODUCT((Expenses!$D$15:$D$103="Travel")*Expenses!$H$15:$H$103)</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="7" t="inlineStr">
+      <c r="B29" s="48" t="inlineStr">
         <is>
           <t>Meals &amp; Entertainment</t>
         </is>
       </c>
       <c r="C29" s="32">
-        <f>SUMPRODUCT((Expenses!$D$4:$D$103="Meals &amp; Entertainment")*Expenses!$F$4:$F$103)</f>
+        <f>SUMPRODUCT((Expenses!$D$4:$D$13="Meals &amp; Entertainment")*Expenses!$F$4:$F$13)+SUMPRODUCT((Expenses!$D$15:$D$103="Meals &amp; Entertainment")*Expenses!$F$15:$F$103)</f>
         <v/>
       </c>
       <c r="D29" s="33">
@@ -4790,18 +4880,18 @@
         <v/>
       </c>
       <c r="E29" s="32">
-        <f>SUMPRODUCT((Expenses!$D$4:$D$103="Meals &amp; Entertainment")*Expenses!$H$4:$H$103)</f>
+        <f>SUMPRODUCT((Expenses!$D$4:$D$13="Meals &amp; Entertainment")*Expenses!$H$4:$H$13)+SUMPRODUCT((Expenses!$D$15:$D$103="Meals &amp; Entertainment")*Expenses!$H$15:$H$103)</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B30" s="47" t="inlineStr">
         <is>
           <t>Professional Services</t>
         </is>
       </c>
       <c r="C30" s="30">
-        <f>SUMPRODUCT((Expenses!$D$4:$D$103="Professional Services")*Expenses!$F$4:$F$103)</f>
+        <f>SUMPRODUCT((Expenses!$D$4:$D$13="Professional Services")*Expenses!$F$4:$F$13)+SUMPRODUCT((Expenses!$D$15:$D$103="Professional Services")*Expenses!$F$15:$F$103)</f>
         <v/>
       </c>
       <c r="D30" s="31">
@@ -4809,18 +4899,18 @@
         <v/>
       </c>
       <c r="E30" s="30">
-        <f>SUMPRODUCT((Expenses!$D$4:$D$103="Professional Services")*Expenses!$H$4:$H$103)</f>
+        <f>SUMPRODUCT((Expenses!$D$4:$D$13="Professional Services")*Expenses!$H$4:$H$13)+SUMPRODUCT((Expenses!$D$15:$D$103="Professional Services")*Expenses!$H$15:$H$103)</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="7" t="inlineStr">
+      <c r="B31" s="48" t="inlineStr">
         <is>
           <t>Marketing &amp; Advertising</t>
         </is>
       </c>
       <c r="C31" s="32">
-        <f>SUMPRODUCT((Expenses!$D$4:$D$103="Marketing &amp; Advertising")*Expenses!$F$4:$F$103)</f>
+        <f>SUMPRODUCT((Expenses!$D$4:$D$13="Marketing &amp; Advertising")*Expenses!$F$4:$F$13)+SUMPRODUCT((Expenses!$D$15:$D$103="Marketing &amp; Advertising")*Expenses!$F$15:$F$103)</f>
         <v/>
       </c>
       <c r="D31" s="33">
@@ -4828,18 +4918,18 @@
         <v/>
       </c>
       <c r="E31" s="32">
-        <f>SUMPRODUCT((Expenses!$D$4:$D$103="Marketing &amp; Advertising")*Expenses!$H$4:$H$103)</f>
+        <f>SUMPRODUCT((Expenses!$D$4:$D$13="Marketing &amp; Advertising")*Expenses!$H$4:$H$13)+SUMPRODUCT((Expenses!$D$15:$D$103="Marketing &amp; Advertising")*Expenses!$H$15:$H$103)</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="B32" s="5" t="inlineStr">
+      <c r="B32" s="47" t="inlineStr">
         <is>
           <t>Insurance</t>
         </is>
       </c>
       <c r="C32" s="30">
-        <f>SUMPRODUCT((Expenses!$D$4:$D$103="Insurance")*Expenses!$F$4:$F$103)</f>
+        <f>SUMPRODUCT((Expenses!$D$4:$D$13="Insurance")*Expenses!$F$4:$F$13)+SUMPRODUCT((Expenses!$D$15:$D$103="Insurance")*Expenses!$F$15:$F$103)</f>
         <v/>
       </c>
       <c r="D32" s="31">
@@ -4847,18 +4937,18 @@
         <v/>
       </c>
       <c r="E32" s="30">
-        <f>SUMPRODUCT((Expenses!$D$4:$D$103="Insurance")*Expenses!$H$4:$H$103)</f>
+        <f>SUMPRODUCT((Expenses!$D$4:$D$13="Insurance")*Expenses!$H$4:$H$13)+SUMPRODUCT((Expenses!$D$15:$D$103="Insurance")*Expenses!$H$15:$H$103)</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="7" t="inlineStr">
+      <c r="B33" s="48" t="inlineStr">
         <is>
           <t>Education &amp; Training</t>
         </is>
       </c>
       <c r="C33" s="32">
-        <f>SUMPRODUCT((Expenses!$D$4:$D$103="Education &amp; Training")*Expenses!$F$4:$F$103)</f>
+        <f>SUMPRODUCT((Expenses!$D$4:$D$13="Education &amp; Training")*Expenses!$F$4:$F$13)+SUMPRODUCT((Expenses!$D$15:$D$103="Education &amp; Training")*Expenses!$F$15:$F$103)</f>
         <v/>
       </c>
       <c r="D33" s="33">
@@ -4866,18 +4956,18 @@
         <v/>
       </c>
       <c r="E33" s="32">
-        <f>SUMPRODUCT((Expenses!$D$4:$D$103="Education &amp; Training")*Expenses!$H$4:$H$103)</f>
+        <f>SUMPRODUCT((Expenses!$D$4:$D$13="Education &amp; Training")*Expenses!$H$4:$H$13)+SUMPRODUCT((Expenses!$D$15:$D$103="Education &amp; Training")*Expenses!$H$15:$H$103)</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="5" t="inlineStr">
+      <c r="B34" s="47" t="inlineStr">
         <is>
           <t>Equipment &amp; Depreciation</t>
         </is>
       </c>
       <c r="C34" s="30">
-        <f>SUMPRODUCT((Expenses!$D$4:$D$103="Equipment &amp; Depreciation")*Expenses!$F$4:$F$103)</f>
+        <f>SUMPRODUCT((Expenses!$D$4:$D$13="Equipment &amp; Depreciation")*Expenses!$F$4:$F$13)+SUMPRODUCT((Expenses!$D$15:$D$103="Equipment &amp; Depreciation")*Expenses!$F$15:$F$103)</f>
         <v/>
       </c>
       <c r="D34" s="31">
@@ -4885,18 +4975,18 @@
         <v/>
       </c>
       <c r="E34" s="30">
-        <f>SUMPRODUCT((Expenses!$D$4:$D$103="Equipment &amp; Depreciation")*Expenses!$H$4:$H$103)</f>
+        <f>SUMPRODUCT((Expenses!$D$4:$D$13="Equipment &amp; Depreciation")*Expenses!$H$4:$H$13)+SUMPRODUCT((Expenses!$D$15:$D$103="Equipment &amp; Depreciation")*Expenses!$H$15:$H$103)</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="7" t="inlineStr">
+      <c r="B35" s="48" t="inlineStr">
         <is>
           <t>Vehicle &amp; Transportation</t>
         </is>
       </c>
       <c r="C35" s="32">
-        <f>SUMPRODUCT((Expenses!$D$4:$D$103="Vehicle &amp; Transportation")*Expenses!$F$4:$F$103)</f>
+        <f>SUMPRODUCT((Expenses!$D$4:$D$13="Vehicle &amp; Transportation")*Expenses!$F$4:$F$13)+SUMPRODUCT((Expenses!$D$15:$D$103="Vehicle &amp; Transportation")*Expenses!$F$15:$F$103)</f>
         <v/>
       </c>
       <c r="D35" s="33">
@@ -4904,18 +4994,18 @@
         <v/>
       </c>
       <c r="E35" s="32">
-        <f>SUMPRODUCT((Expenses!$D$4:$D$103="Vehicle &amp; Transportation")*Expenses!$H$4:$H$103)</f>
+        <f>SUMPRODUCT((Expenses!$D$4:$D$13="Vehicle &amp; Transportation")*Expenses!$H$4:$H$13)+SUMPRODUCT((Expenses!$D$15:$D$103="Vehicle &amp; Transportation")*Expenses!$H$15:$H$103)</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="5" t="inlineStr">
+      <c r="B36" s="47" t="inlineStr">
         <is>
           <t>Bank Fees &amp; Interest</t>
         </is>
       </c>
       <c r="C36" s="30">
-        <f>SUMPRODUCT((Expenses!$D$4:$D$103="Bank Fees &amp; Interest")*Expenses!$F$4:$F$103)</f>
+        <f>SUMPRODUCT((Expenses!$D$4:$D$13="Bank Fees &amp; Interest")*Expenses!$F$4:$F$13)+SUMPRODUCT((Expenses!$D$15:$D$103="Bank Fees &amp; Interest")*Expenses!$F$15:$F$103)</f>
         <v/>
       </c>
       <c r="D36" s="31">
@@ -4923,18 +5013,18 @@
         <v/>
       </c>
       <c r="E36" s="30">
-        <f>SUMPRODUCT((Expenses!$D$4:$D$103="Bank Fees &amp; Interest")*Expenses!$H$4:$H$103)</f>
+        <f>SUMPRODUCT((Expenses!$D$4:$D$13="Bank Fees &amp; Interest")*Expenses!$H$4:$H$13)+SUMPRODUCT((Expenses!$D$15:$D$103="Bank Fees &amp; Interest")*Expenses!$H$15:$H$103)</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="7" t="inlineStr">
+      <c r="B37" s="48" t="inlineStr">
         <is>
           <t>Taxes &amp; Licenses</t>
         </is>
       </c>
       <c r="C37" s="32">
-        <f>SUMPRODUCT((Expenses!$D$4:$D$103="Taxes &amp; Licenses")*Expenses!$F$4:$F$103)</f>
+        <f>SUMPRODUCT((Expenses!$D$4:$D$13="Taxes &amp; Licenses")*Expenses!$F$4:$F$13)+SUMPRODUCT((Expenses!$D$15:$D$103="Taxes &amp; Licenses")*Expenses!$F$15:$F$103)</f>
         <v/>
       </c>
       <c r="D37" s="33">
@@ -4942,31 +5032,31 @@
         <v/>
       </c>
       <c r="E37" s="32">
-        <f>SUMPRODUCT((Expenses!$D$4:$D$103="Taxes &amp; Licenses")*Expenses!$H$4:$H$103)</f>
+        <f>SUMPRODUCT((Expenses!$D$4:$D$13="Taxes &amp; Licenses")*Expenses!$H$4:$H$13)+SUMPRODUCT((Expenses!$D$15:$D$103="Taxes &amp; Licenses")*Expenses!$H$15:$H$103)</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="28" t="inlineStr">
+      <c r="B38" s="45" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C38" s="29">
+      <c r="C38" s="46">
+        <f>SUM(C26:C37)</f>
+        <v/>
+      </c>
+      <c r="D38" s="49">
         <f>SUM(D26:D37)</f>
         <v/>
       </c>
-      <c r="D38" s="34">
+      <c r="E38" s="46">
         <f>SUM(E26:E37)</f>
         <v/>
       </c>
-      <c r="E38" s="29">
-        <f>SUM(F26:F37)</f>
-        <v/>
-      </c>
     </row>
     <row r="40">
-      <c r="B40" s="27" t="inlineStr">
+      <c r="B40" s="43" t="inlineStr">
         <is>
           <t>Top Clients by Revenue</t>
         </is>
@@ -4976,30 +5066,29 @@
       <c r="E40" s="17" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="12" t="n"/>
-      <c r="B41" s="12" t="inlineStr">
+      <c r="B41" s="44" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
-      <c r="C41" s="12" t="inlineStr">
+      <c r="C41" s="44" t="inlineStr">
         <is>
           <t>Total Revenue</t>
         </is>
       </c>
-      <c r="D41" s="12" t="inlineStr">
+      <c r="D41" s="44" t="inlineStr">
         <is>
           <t># Invoices</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E41" s="44" t="inlineStr">
         <is>
           <t>Avg per Invoice</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="5" t="inlineStr">
+      <c r="B42" s="47" t="inlineStr">
         <is>
           <t>Acme Corp</t>
         </is>
@@ -5018,7 +5107,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="B43" s="7" t="inlineStr">
+      <c r="B43" s="48" t="inlineStr">
         <is>
           <t>TechStart Inc</t>
         </is>
@@ -5037,7 +5126,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="B44" s="5" t="inlineStr">
+      <c r="B44" s="47" t="inlineStr">
         <is>
           <t>MediaCo</t>
         </is>
@@ -5056,7 +5145,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="B45" s="7" t="inlineStr">
+      <c r="B45" s="48" t="inlineStr">
         <is>
           <t>LocalShop</t>
         </is>
@@ -5075,7 +5164,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="B47" s="27" t="inlineStr">
+      <c r="B47" s="43" t="inlineStr">
         <is>
           <t>2026 Quarterly Tax Payment Schedule</t>
         </is>
@@ -5086,35 +5175,34 @@
       <c r="F47" s="17" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="12" t="n"/>
-      <c r="B48" s="12" t="inlineStr">
+      <c r="B48" s="44" t="inlineStr">
         <is>
           <t>Quarter</t>
         </is>
       </c>
-      <c r="C48" s="12" t="inlineStr">
+      <c r="C48" s="44" t="inlineStr">
         <is>
           <t>Deadline</t>
         </is>
       </c>
-      <c r="D48" s="12" t="inlineStr">
+      <c r="D48" s="44" t="inlineStr">
         <is>
           <t>Payment Due</t>
         </is>
       </c>
-      <c r="E48" s="12" t="inlineStr">
+      <c r="E48" s="44" t="inlineStr">
         <is>
           <t>Income Period</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F48" s="44" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="B49" s="5" t="inlineStr">
+      <c r="B49" s="47" t="inlineStr">
         <is>
           <t>Q1</t>
         </is>
@@ -5125,7 +5213,7 @@
         </is>
       </c>
       <c r="D49" s="14">
-        <f>B8/4</f>
+        <f>G5/4</f>
         <v/>
       </c>
       <c r="E49" s="6" t="inlineStr">
@@ -5140,7 +5228,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="B50" s="7" t="inlineStr">
+      <c r="B50" s="48" t="inlineStr">
         <is>
           <t>Q2</t>
         </is>
@@ -5151,7 +5239,7 @@
         </is>
       </c>
       <c r="D50" s="16">
-        <f>B8/4</f>
+        <f>G5/4</f>
         <v/>
       </c>
       <c r="E50" s="8" t="inlineStr">
@@ -5166,7 +5254,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="B51" s="5" t="inlineStr">
+      <c r="B51" s="47" t="inlineStr">
         <is>
           <t>Q3</t>
         </is>
@@ -5177,7 +5265,7 @@
         </is>
       </c>
       <c r="D51" s="14">
-        <f>B8/4</f>
+        <f>G5/4</f>
         <v/>
       </c>
       <c r="E51" s="6" t="inlineStr">
@@ -5192,7 +5280,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="B52" s="7" t="inlineStr">
+      <c r="B52" s="48" t="inlineStr">
         <is>
           <t>Q4</t>
         </is>
@@ -5203,7 +5291,7 @@
         </is>
       </c>
       <c r="D52" s="16">
-        <f>B8/4</f>
+        <f>G5/4</f>
         <v/>
       </c>
       <c r="E52" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Fix platform fee column - default to 0, not 5%
</commit_message>
<xml_diff>
--- a/Freelancer_Finance_Dashboard.xlsx
+++ b/Freelancer_Finance_Dashboard.xlsx
@@ -1069,9 +1069,8 @@
       <c r="F4" s="14" t="n">
         <v>5000</v>
       </c>
-      <c r="G4" s="14">
-        <f>IF(F4="","",F4*0.05)</f>
-        <v/>
+      <c r="G4" s="14" t="n">
+        <v>0</v>
       </c>
       <c r="H4" s="14">
         <f>F4-G4</f>
@@ -1110,9 +1109,8 @@
       <c r="F5" s="16" t="n">
         <v>3500</v>
       </c>
-      <c r="G5" s="16">
-        <f>IF(F5="","",F5*0.05)</f>
-        <v/>
+      <c r="G5" s="16" t="n">
+        <v>175</v>
       </c>
       <c r="H5" s="16">
         <f>F5-G5</f>
@@ -1151,9 +1149,8 @@
       <c r="F6" s="14" t="n">
         <v>5000</v>
       </c>
-      <c r="G6" s="14">
-        <f>IF(F6="","",F6*0.05)</f>
-        <v/>
+      <c r="G6" s="14" t="n">
+        <v>0</v>
       </c>
       <c r="H6" s="14">
         <f>F6-G6</f>
@@ -1192,9 +1189,8 @@
       <c r="F7" s="16" t="n">
         <v>2800</v>
       </c>
-      <c r="G7" s="16">
-        <f>IF(F7="","",F7*0.05)</f>
-        <v/>
+      <c r="G7" s="16" t="n">
+        <v>140</v>
       </c>
       <c r="H7" s="16">
         <f>F7-G7</f>
@@ -1233,9 +1229,8 @@
       <c r="F8" s="14" t="n">
         <v>1500</v>
       </c>
-      <c r="G8" s="14">
-        <f>IF(F8="","",F8*0.05)</f>
-        <v/>
+      <c r="G8" s="14" t="n">
+        <v>0</v>
       </c>
       <c r="H8" s="14">
         <f>F8-G8</f>
@@ -1282,7 +1277,7 @@
       <c r="E10" s="8" t="n"/>
       <c r="F10" s="16" t="n"/>
       <c r="G10" s="16">
-        <f>IF(F10="","",F10*0.05)</f>
+        <f>IF(F10="","",0)</f>
         <v/>
       </c>
       <c r="H10" s="16">
@@ -1302,7 +1297,7 @@
       <c r="E11" s="8" t="n"/>
       <c r="F11" s="16" t="n"/>
       <c r="G11" s="16">
-        <f>IF(F11="","",F11*0.05)</f>
+        <f>IF(F11="","",0)</f>
         <v/>
       </c>
       <c r="H11" s="16">
@@ -1322,7 +1317,7 @@
       <c r="E12" s="8" t="n"/>
       <c r="F12" s="16" t="n"/>
       <c r="G12" s="16">
-        <f>IF(F12="","",F12*0.05)</f>
+        <f>IF(F12="","",0)</f>
         <v/>
       </c>
       <c r="H12" s="16">
@@ -1342,7 +1337,7 @@
       <c r="E13" s="8" t="n"/>
       <c r="F13" s="16" t="n"/>
       <c r="G13" s="16">
-        <f>IF(F13="","",F13*0.05)</f>
+        <f>IF(F13="","",0)</f>
         <v/>
       </c>
       <c r="H13" s="16">
@@ -1362,7 +1357,7 @@
       <c r="E14" s="8" t="n"/>
       <c r="F14" s="16" t="n"/>
       <c r="G14" s="16">
-        <f>IF(F14="","",F14*0.05)</f>
+        <f>IF(F14="","",0)</f>
         <v/>
       </c>
       <c r="H14" s="16">
@@ -1382,7 +1377,7 @@
       <c r="E15" s="8" t="n"/>
       <c r="F15" s="16" t="n"/>
       <c r="G15" s="16">
-        <f>IF(F15="","",F15*0.05)</f>
+        <f>IF(F15="","",0)</f>
         <v/>
       </c>
       <c r="H15" s="16">
@@ -1402,7 +1397,7 @@
       <c r="E16" s="8" t="n"/>
       <c r="F16" s="16" t="n"/>
       <c r="G16" s="16">
-        <f>IF(F16="","",F16*0.05)</f>
+        <f>IF(F16="","",0)</f>
         <v/>
       </c>
       <c r="H16" s="16">
@@ -1422,7 +1417,7 @@
       <c r="E17" s="8" t="n"/>
       <c r="F17" s="16" t="n"/>
       <c r="G17" s="16">
-        <f>IF(F17="","",F17*0.05)</f>
+        <f>IF(F17="","",0)</f>
         <v/>
       </c>
       <c r="H17" s="16">
@@ -1442,7 +1437,7 @@
       <c r="E18" s="8" t="n"/>
       <c r="F18" s="16" t="n"/>
       <c r="G18" s="16">
-        <f>IF(F18="","",F18*0.05)</f>
+        <f>IF(F18="","",0)</f>
         <v/>
       </c>
       <c r="H18" s="16">
@@ -1462,7 +1457,7 @@
       <c r="E19" s="8" t="n"/>
       <c r="F19" s="16" t="n"/>
       <c r="G19" s="16">
-        <f>IF(F19="","",F19*0.05)</f>
+        <f>IF(F19="","",0)</f>
         <v/>
       </c>
       <c r="H19" s="16">
@@ -1482,7 +1477,7 @@
       <c r="E20" s="8" t="n"/>
       <c r="F20" s="16" t="n"/>
       <c r="G20" s="16">
-        <f>IF(F20="","",F20*0.05)</f>
+        <f>IF(F20="","",0)</f>
         <v/>
       </c>
       <c r="H20" s="16">
@@ -1502,7 +1497,7 @@
       <c r="E21" s="8" t="n"/>
       <c r="F21" s="16" t="n"/>
       <c r="G21" s="16">
-        <f>IF(F21="","",F21*0.05)</f>
+        <f>IF(F21="","",0)</f>
         <v/>
       </c>
       <c r="H21" s="16">
@@ -1522,7 +1517,7 @@
       <c r="E22" s="8" t="n"/>
       <c r="F22" s="16" t="n"/>
       <c r="G22" s="16">
-        <f>IF(F22="","",F22*0.05)</f>
+        <f>IF(F22="","",0)</f>
         <v/>
       </c>
       <c r="H22" s="16">
@@ -1542,7 +1537,7 @@
       <c r="E23" s="8" t="n"/>
       <c r="F23" s="16" t="n"/>
       <c r="G23" s="16">
-        <f>IF(F23="","",F23*0.05)</f>
+        <f>IF(F23="","",0)</f>
         <v/>
       </c>
       <c r="H23" s="16">
@@ -1562,7 +1557,7 @@
       <c r="E24" s="8" t="n"/>
       <c r="F24" s="16" t="n"/>
       <c r="G24" s="16">
-        <f>IF(F24="","",F24*0.05)</f>
+        <f>IF(F24="","",0)</f>
         <v/>
       </c>
       <c r="H24" s="16">
@@ -1582,7 +1577,7 @@
       <c r="E25" s="8" t="n"/>
       <c r="F25" s="16" t="n"/>
       <c r="G25" s="16">
-        <f>IF(F25="","",F25*0.05)</f>
+        <f>IF(F25="","",0)</f>
         <v/>
       </c>
       <c r="H25" s="16">
@@ -1602,7 +1597,7 @@
       <c r="E26" s="8" t="n"/>
       <c r="F26" s="16" t="n"/>
       <c r="G26" s="16">
-        <f>IF(F26="","",F26*0.05)</f>
+        <f>IF(F26="","",0)</f>
         <v/>
       </c>
       <c r="H26" s="16">
@@ -1622,7 +1617,7 @@
       <c r="E27" s="8" t="n"/>
       <c r="F27" s="16" t="n"/>
       <c r="G27" s="16">
-        <f>IF(F27="","",F27*0.05)</f>
+        <f>IF(F27="","",0)</f>
         <v/>
       </c>
       <c r="H27" s="16">
@@ -1642,7 +1637,7 @@
       <c r="E28" s="8" t="n"/>
       <c r="F28" s="16" t="n"/>
       <c r="G28" s="16">
-        <f>IF(F28="","",F28*0.05)</f>
+        <f>IF(F28="","",0)</f>
         <v/>
       </c>
       <c r="H28" s="16">
@@ -1662,7 +1657,7 @@
       <c r="E29" s="8" t="n"/>
       <c r="F29" s="16" t="n"/>
       <c r="G29" s="16">
-        <f>IF(F29="","",F29*0.05)</f>
+        <f>IF(F29="","",0)</f>
         <v/>
       </c>
       <c r="H29" s="16">
@@ -1682,7 +1677,7 @@
       <c r="E30" s="8" t="n"/>
       <c r="F30" s="16" t="n"/>
       <c r="G30" s="16">
-        <f>IF(F30="","",F30*0.05)</f>
+        <f>IF(F30="","",0)</f>
         <v/>
       </c>
       <c r="H30" s="16">
@@ -1702,7 +1697,7 @@
       <c r="E31" s="8" t="n"/>
       <c r="F31" s="16" t="n"/>
       <c r="G31" s="16">
-        <f>IF(F31="","",F31*0.05)</f>
+        <f>IF(F31="","",0)</f>
         <v/>
       </c>
       <c r="H31" s="16">
@@ -1722,7 +1717,7 @@
       <c r="E32" s="8" t="n"/>
       <c r="F32" s="16" t="n"/>
       <c r="G32" s="16">
-        <f>IF(F32="","",F32*0.05)</f>
+        <f>IF(F32="","",0)</f>
         <v/>
       </c>
       <c r="H32" s="16">
@@ -1742,7 +1737,7 @@
       <c r="E33" s="8" t="n"/>
       <c r="F33" s="16" t="n"/>
       <c r="G33" s="16">
-        <f>IF(F33="","",F33*0.05)</f>
+        <f>IF(F33="","",0)</f>
         <v/>
       </c>
       <c r="H33" s="16">
@@ -1762,7 +1757,7 @@
       <c r="E34" s="8" t="n"/>
       <c r="F34" s="16" t="n"/>
       <c r="G34" s="16">
-        <f>IF(F34="","",F34*0.05)</f>
+        <f>IF(F34="","",0)</f>
         <v/>
       </c>
       <c r="H34" s="16">
@@ -1782,7 +1777,7 @@
       <c r="E35" s="8" t="n"/>
       <c r="F35" s="16" t="n"/>
       <c r="G35" s="16">
-        <f>IF(F35="","",F35*0.05)</f>
+        <f>IF(F35="","",0)</f>
         <v/>
       </c>
       <c r="H35" s="16">
@@ -1802,7 +1797,7 @@
       <c r="E36" s="8" t="n"/>
       <c r="F36" s="16" t="n"/>
       <c r="G36" s="16">
-        <f>IF(F36="","",F36*0.05)</f>
+        <f>IF(F36="","",0)</f>
         <v/>
       </c>
       <c r="H36" s="16">
@@ -1822,7 +1817,7 @@
       <c r="E37" s="8" t="n"/>
       <c r="F37" s="16" t="n"/>
       <c r="G37" s="16">
-        <f>IF(F37="","",F37*0.05)</f>
+        <f>IF(F37="","",0)</f>
         <v/>
       </c>
       <c r="H37" s="16">
@@ -1842,7 +1837,7 @@
       <c r="E38" s="8" t="n"/>
       <c r="F38" s="16" t="n"/>
       <c r="G38" s="16">
-        <f>IF(F38="","",F38*0.05)</f>
+        <f>IF(F38="","",0)</f>
         <v/>
       </c>
       <c r="H38" s="16">
@@ -1862,7 +1857,7 @@
       <c r="E39" s="8" t="n"/>
       <c r="F39" s="16" t="n"/>
       <c r="G39" s="16">
-        <f>IF(F39="","",F39*0.05)</f>
+        <f>IF(F39="","",0)</f>
         <v/>
       </c>
       <c r="H39" s="16">
@@ -1882,7 +1877,7 @@
       <c r="E40" s="8" t="n"/>
       <c r="F40" s="16" t="n"/>
       <c r="G40" s="16">
-        <f>IF(F40="","",F40*0.05)</f>
+        <f>IF(F40="","",0)</f>
         <v/>
       </c>
       <c r="H40" s="16">
@@ -1902,7 +1897,7 @@
       <c r="E41" s="8" t="n"/>
       <c r="F41" s="16" t="n"/>
       <c r="G41" s="16">
-        <f>IF(F41="","",F41*0.05)</f>
+        <f>IF(F41="","",0)</f>
         <v/>
       </c>
       <c r="H41" s="16">
@@ -1922,7 +1917,7 @@
       <c r="E42" s="8" t="n"/>
       <c r="F42" s="16" t="n"/>
       <c r="G42" s="16">
-        <f>IF(F42="","",F42*0.05)</f>
+        <f>IF(F42="","",0)</f>
         <v/>
       </c>
       <c r="H42" s="16">
@@ -1942,7 +1937,7 @@
       <c r="E43" s="8" t="n"/>
       <c r="F43" s="16" t="n"/>
       <c r="G43" s="16">
-        <f>IF(F43="","",F43*0.05)</f>
+        <f>IF(F43="","",0)</f>
         <v/>
       </c>
       <c r="H43" s="16">
@@ -1962,7 +1957,7 @@
       <c r="E44" s="8" t="n"/>
       <c r="F44" s="16" t="n"/>
       <c r="G44" s="16">
-        <f>IF(F44="","",F44*0.05)</f>
+        <f>IF(F44="","",0)</f>
         <v/>
       </c>
       <c r="H44" s="16">
@@ -1982,7 +1977,7 @@
       <c r="E45" s="8" t="n"/>
       <c r="F45" s="16" t="n"/>
       <c r="G45" s="16">
-        <f>IF(F45="","",F45*0.05)</f>
+        <f>IF(F45="","",0)</f>
         <v/>
       </c>
       <c r="H45" s="16">
@@ -2002,7 +1997,7 @@
       <c r="E46" s="8" t="n"/>
       <c r="F46" s="16" t="n"/>
       <c r="G46" s="16">
-        <f>IF(F46="","",F46*0.05)</f>
+        <f>IF(F46="","",0)</f>
         <v/>
       </c>
       <c r="H46" s="16">
@@ -2022,7 +2017,7 @@
       <c r="E47" s="8" t="n"/>
       <c r="F47" s="16" t="n"/>
       <c r="G47" s="16">
-        <f>IF(F47="","",F47*0.05)</f>
+        <f>IF(F47="","",0)</f>
         <v/>
       </c>
       <c r="H47" s="16">
@@ -2042,7 +2037,7 @@
       <c r="E48" s="8" t="n"/>
       <c r="F48" s="16" t="n"/>
       <c r="G48" s="16">
-        <f>IF(F48="","",F48*0.05)</f>
+        <f>IF(F48="","",0)</f>
         <v/>
       </c>
       <c r="H48" s="16">
@@ -2062,7 +2057,7 @@
       <c r="E49" s="8" t="n"/>
       <c r="F49" s="16" t="n"/>
       <c r="G49" s="16">
-        <f>IF(F49="","",F49*0.05)</f>
+        <f>IF(F49="","",0)</f>
         <v/>
       </c>
       <c r="H49" s="16">
@@ -2082,7 +2077,7 @@
       <c r="E50" s="8" t="n"/>
       <c r="F50" s="16" t="n"/>
       <c r="G50" s="16">
-        <f>IF(F50="","",F50*0.05)</f>
+        <f>IF(F50="","",0)</f>
         <v/>
       </c>
       <c r="H50" s="16">
@@ -2102,7 +2097,7 @@
       <c r="E51" s="8" t="n"/>
       <c r="F51" s="16" t="n"/>
       <c r="G51" s="16">
-        <f>IF(F51="","",F51*0.05)</f>
+        <f>IF(F51="","",0)</f>
         <v/>
       </c>
       <c r="H51" s="16">
@@ -2122,7 +2117,7 @@
       <c r="E52" s="8" t="n"/>
       <c r="F52" s="16" t="n"/>
       <c r="G52" s="16">
-        <f>IF(F52="","",F52*0.05)</f>
+        <f>IF(F52="","",0)</f>
         <v/>
       </c>
       <c r="H52" s="16">
@@ -2142,7 +2137,7 @@
       <c r="E53" s="8" t="n"/>
       <c r="F53" s="16" t="n"/>
       <c r="G53" s="16">
-        <f>IF(F53="","",F53*0.05)</f>
+        <f>IF(F53="","",0)</f>
         <v/>
       </c>
       <c r="H53" s="16">

</xml_diff>